<commit_message>
Add g=0.95 data for n=1.8 ETL/HTL 500 nm case
New BSDF slice (S=1:2:15, g=0.95, n_SL=1.8) and its sweep result,
merged into the raw-data spreadsheet between g=0.9 and g=1.0.
EQE plateaus at 0.80-0.81 for S>=5 (max 0.8096 at S=11); S=1 is
under-scattered (S'=0.05, EQE 0.68).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0138cXdpoaC96Qa968PD6P1C
</commit_message>
<xml_diff>
--- a/EQE_SL_raw_data_S_vs_g.xlsx
+++ b/EQE_SL_raw_data_S_vs_g.xlsx
@@ -639,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -658,6 +658,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -680,6 +681,9 @@
         <v>0.9</v>
       </c>
       <c r="G3" s="5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H3" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -703,6 +707,9 @@
         <v>0.753881</v>
       </c>
       <c r="G4" s="6" t="n">
+        <v>0.679825</v>
+      </c>
+      <c r="H4" s="6" t="n">
         <v>0.206945</v>
       </c>
     </row>
@@ -726,6 +733,9 @@
         <v>0.804253</v>
       </c>
       <c r="G5" s="6" t="n">
+        <v>0.784639</v>
+      </c>
+      <c r="H5" s="6" t="n">
         <v>0.206942</v>
       </c>
     </row>
@@ -749,6 +759,9 @@
         <v>0.809096</v>
       </c>
       <c r="G6" s="6" t="n">
+        <v>0.80163</v>
+      </c>
+      <c r="H6" s="6" t="n">
         <v>0.206943</v>
       </c>
     </row>
@@ -772,6 +785,9 @@
         <v>0.808132</v>
       </c>
       <c r="G7" s="6" t="n">
+        <v>0.807364</v>
+      </c>
+      <c r="H7" s="6" t="n">
         <v>0.206948</v>
       </c>
     </row>
@@ -795,6 +811,9 @@
         <v>0.805727</v>
       </c>
       <c r="G8" s="6" t="n">
+        <v>0.809157</v>
+      </c>
+      <c r="H8" s="6" t="n">
         <v>0.20694</v>
       </c>
     </row>
@@ -818,6 +837,9 @@
         <v>0.80248</v>
       </c>
       <c r="G9" s="6" t="n">
+        <v>0.809593</v>
+      </c>
+      <c r="H9" s="6" t="n">
         <v>0.20694</v>
       </c>
     </row>
@@ -841,6 +863,9 @@
         <v>0.798996</v>
       </c>
       <c r="G10" s="6" t="n">
+        <v>0.808812</v>
+      </c>
+      <c r="H10" s="6" t="n">
         <v>0.206939</v>
       </c>
     </row>
@@ -864,6 +889,9 @@
         <v>0.7955179999999999</v>
       </c>
       <c r="G11" s="6" t="n">
+        <v>0.807827</v>
+      </c>
+      <c r="H11" s="6" t="n">
         <v>0.206943</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add n=1.51 ETL/HTL 500 nm sweep (same S,g range incl. g=0.95)
Planar EQE_air = 0.213, EQE_sub = 0.565. Scattering layer gives
0.446-0.533; plateau ~0.53 for S(1-g) in 0.3-3 (max 0.5325 at
S=9, g=0.95). Results merged into the raw-data spreadsheet as
sheet n1.51_ETLHTL500.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0138cXdpoaC96Qa968PD6P1C
</commit_message>
<xml_diff>
--- a/EQE_SL_raw_data_S_vs_g.xlsx
+++ b/EQE_SL_raw_data_S_vs_g.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="n1.80_ETLHTL500" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="n1.80_ETLHTL80" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="n1.51_ETLHTL80" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="n1.51_ETLHTL150" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="n1.51_ETLHTL200" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="n1.51_ETLHTL500" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="n1.80_ETLHTL80" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="n1.51_ETLHTL80" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="n1.51_ETLHTL150" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="n1.51_ETLHTL200" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -445,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -559,72 +560,90 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>n1.80_ETLHTL80</t>
+          <t>n1.51_ETLHTL500</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
+          <t>n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.1854</v>
+        <v>0.2126</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.8097</v>
+        <v>0.5649</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL80</t>
+          <t>n1.80_ETLHTL80</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
+          <t>n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.1865</v>
+        <v>0.1854</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.5525</v>
+        <v>0.8097</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>n1.51_ETLHTL150</t>
+          <t>n1.51_ETLHTL80</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+          <t>n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.1311</v>
+        <v>0.1865</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.4005</v>
+        <v>0.5525</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>n1.51_ETLHTL150</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>0.1311</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>0.4005</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>n1.51_ETLHTL200</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>n_sub = n_SL = 1.51, ETL 200 nm / HTL 200 nm x3</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C14" s="2" t="n">
         <v>0.3347</v>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D14" s="2" t="n">
         <v>0.5671</v>
       </c>
     </row>
@@ -658,7 +677,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -906,7 +924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -916,12 +934,13 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL(B3) 500 nm / HTL(TAPC) 500 nm x3</t>
         </is>
       </c>
     </row>
@@ -947,6 +966,9 @@
         <v>0.9</v>
       </c>
       <c r="G3" s="5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H3" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -955,22 +977,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.721296</v>
+        <v>0.530174</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.720206</v>
+        <v>0.530294</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.716857</v>
+        <v>0.529574</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.707013</v>
+        <v>0.526768</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.672125</v>
+        <v>0.515456</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.182393</v>
+        <v>0.489715</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>0.206753</v>
       </c>
     </row>
     <row r="5">
@@ -978,22 +1003,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.716266</v>
+        <v>0.522313</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.721016</v>
+        <v>0.525689</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.725425</v>
+        <v>0.528843</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.728177</v>
+        <v>0.531454</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.723059</v>
+        <v>0.531369</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.182389</v>
+        <v>0.5251749999999999</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0.206749</v>
       </c>
     </row>
     <row r="6">
@@ -1001,22 +1029,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.698484</v>
+        <v>0.510482</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.707616</v>
+        <v>0.516444</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.716408</v>
+        <v>0.522269</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.724815</v>
+        <v>0.527867</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.72904</v>
+        <v>0.532183</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.182388</v>
+        <v>0.530655</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.206749</v>
       </c>
     </row>
     <row r="7">
@@ -1024,22 +1055,25 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.6793630000000001</v>
+        <v>0.498234</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.692587</v>
+        <v>0.506833</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.705593</v>
+        <v>0.515134</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.718198</v>
+        <v>0.523386</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.728581</v>
+        <v>0.530869</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.182403</v>
+        <v>0.532184</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0.206748</v>
       </c>
     </row>
     <row r="8">
@@ -1047,22 +1081,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.660434</v>
+        <v>0.485254</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.677283</v>
+        <v>0.496809</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.694479</v>
+        <v>0.507911</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.7111769999999999</v>
+        <v>0.51874</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.726436</v>
+        <v>0.528961</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.182386</v>
+        <v>0.532516</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0.206749</v>
       </c>
     </row>
     <row r="9">
@@ -1070,22 +1107,25 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.64097</v>
+        <v>0.472283</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.662505</v>
+        <v>0.486424</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.6832780000000001</v>
+        <v>0.500487</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.703989</v>
+        <v>0.513952</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.723368</v>
+        <v>0.526794</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.182387</v>
+        <v>0.5321050000000001</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0.206748</v>
       </c>
     </row>
     <row r="10">
@@ -1093,22 +1133,25 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.622152</v>
+        <v>0.459081</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.6469510000000001</v>
+        <v>0.476091</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.671573</v>
+        <v>0.492779</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.696204</v>
+        <v>0.509009</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.719983</v>
+        <v>0.524493</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.182385</v>
+        <v>0.531368</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.206748</v>
       </c>
     </row>
     <row r="11">
@@ -1116,22 +1159,25 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.604131</v>
+        <v>0.445793</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.631347</v>
+        <v>0.465539</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.659758</v>
+        <v>0.4851</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.68865</v>
+        <v>0.504113</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.716566</v>
+        <v>0.522168</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.182391</v>
+        <v>0.53046</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0.206747</v>
       </c>
     </row>
   </sheetData>
@@ -1160,7 +1206,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.80, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
     </row>
@@ -1194,22 +1240,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.51635</v>
+        <v>0.721296</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.516308</v>
+        <v>0.720206</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.515298</v>
+        <v>0.716857</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.511908</v>
+        <v>0.707013</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.499114</v>
+        <v>0.672125</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.177993</v>
+        <v>0.182393</v>
       </c>
     </row>
     <row r="5">
@@ -1217,22 +1263,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.509284</v>
+        <v>0.716266</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.512656</v>
+        <v>0.721016</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.515756</v>
+        <v>0.725425</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.518181</v>
+        <v>0.728177</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.517415</v>
+        <v>0.723059</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.17799</v>
+        <v>0.182389</v>
       </c>
     </row>
     <row r="6">
@@ -1240,22 +1286,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.497442</v>
+        <v>0.698484</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.5034380000000001</v>
+        <v>0.707616</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.509286</v>
+        <v>0.716408</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.514854</v>
+        <v>0.724815</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.51884</v>
+        <v>0.72904</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.17799</v>
+        <v>0.182388</v>
       </c>
     </row>
     <row r="7">
@@ -1263,22 +1309,22 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.485185</v>
+        <v>0.6793630000000001</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.493792</v>
+        <v>0.692587</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.502116</v>
+        <v>0.705593</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.510412</v>
+        <v>0.718198</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.517763</v>
+        <v>0.728581</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.177988</v>
+        <v>0.182403</v>
       </c>
     </row>
     <row r="8">
@@ -1286,22 +1332,22 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.472241</v>
+        <v>0.660434</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.483754</v>
+        <v>0.677283</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.494866</v>
+        <v>0.694479</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.505745</v>
+        <v>0.7111769999999999</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.515954</v>
+        <v>0.726436</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.182386</v>
       </c>
     </row>
     <row r="9">
@@ -1309,22 +1355,22 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.459365</v>
+        <v>0.64097</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.473397</v>
+        <v>0.662505</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.487421</v>
+        <v>0.6832780000000001</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.50093</v>
+        <v>0.703989</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.513819</v>
+        <v>0.723368</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.182387</v>
       </c>
     </row>
     <row r="10">
@@ -1332,22 +1378,22 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.446312</v>
+        <v>0.622152</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.463127</v>
+        <v>0.6469510000000001</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.479721</v>
+        <v>0.671573</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.495954</v>
+        <v>0.696204</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.511526</v>
+        <v>0.719983</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.177989</v>
+        <v>0.182385</v>
       </c>
     </row>
     <row r="11">
@@ -1355,22 +1401,22 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.433206</v>
+        <v>0.604131</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.452681</v>
+        <v>0.631347</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.472072</v>
+        <v>0.659758</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.491045</v>
+        <v>0.68865</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.509188</v>
+        <v>0.716566</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.177987</v>
+        <v>0.182391</v>
       </c>
     </row>
   </sheetData>
@@ -1399,7 +1445,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 80 nm / HTL 80 nm x3</t>
         </is>
       </c>
     </row>
@@ -1433,22 +1479,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.375381</v>
+        <v>0.51635</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>0.375408</v>
+        <v>0.516308</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.374819</v>
+        <v>0.515298</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.372681</v>
+        <v>0.511908</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>0.364118</v>
+        <v>0.499114</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.128306</v>
+        <v>0.177993</v>
       </c>
     </row>
     <row r="5">
@@ -1456,22 +1502,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.369639</v>
+        <v>0.509284</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.371995</v>
+        <v>0.512656</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.374193</v>
+        <v>0.515756</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.376003</v>
+        <v>0.518181</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.375864</v>
+        <v>0.517415</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.128304</v>
+        <v>0.17799</v>
       </c>
     </row>
     <row r="6">
@@ -1479,22 +1525,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.361244</v>
+        <v>0.497442</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.365423</v>
+        <v>0.5034380000000001</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.369509</v>
+        <v>0.509286</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.373419</v>
+        <v>0.514854</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.376431</v>
+        <v>0.51884</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.17799</v>
       </c>
     </row>
     <row r="7">
@@ -1502,22 +1548,22 @@
         <v>7</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.352561</v>
+        <v>0.485185</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.358622</v>
+        <v>0.493792</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.364454</v>
+        <v>0.502116</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.370239</v>
+        <v>0.510412</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.375481</v>
+        <v>0.517763</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.128302</v>
+        <v>0.177988</v>
       </c>
     </row>
     <row r="8">
@@ -1525,22 +1571,22 @@
         <v>9</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.343355</v>
+        <v>0.472241</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.351511</v>
+        <v>0.483754</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.359337</v>
+        <v>0.494866</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.366944</v>
+        <v>0.505745</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.374115</v>
+        <v>0.515954</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.177989</v>
       </c>
     </row>
     <row r="9">
@@ -1548,22 +1594,22 @@
         <v>11</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.334158</v>
+        <v>0.459365</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.344156</v>
+        <v>0.473397</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.354078</v>
+        <v>0.487421</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.363558</v>
+        <v>0.50093</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.372577</v>
+        <v>0.513819</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.177989</v>
       </c>
     </row>
     <row r="10">
@@ -1571,22 +1617,22 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.324795</v>
+        <v>0.446312</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.336824</v>
+        <v>0.463127</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.348606</v>
+        <v>0.479721</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.360058</v>
+        <v>0.495954</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.370937</v>
+        <v>0.511526</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.128303</v>
+        <v>0.177989</v>
       </c>
     </row>
     <row r="11">
@@ -1594,22 +1640,22 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.315368</v>
+        <v>0.433206</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.329339</v>
+        <v>0.452681</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.343169</v>
+        <v>0.472072</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.356587</v>
+        <v>0.491045</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.369291</v>
+        <v>0.509188</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.128302</v>
+        <v>0.177987</v>
       </c>
     </row>
   </sheetData>
@@ -1638,6 +1684,245 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
+          <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 150 nm / HTL 150 nm x3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>S \ g</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>0.375381</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>0.375408</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0.374819</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>0.372681</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>0.364118</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0.128306</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0.369639</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0.371995</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0.374193</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0.376003</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0.375864</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0.128304</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>0.361244</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.365423</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0.369509</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.373419</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>0.376431</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>0.352561</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.358622</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.364454</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0.370239</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.375481</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0.128302</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>0.343355</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.351511</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0.359337</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>0.366944</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0.374115</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>0.334158</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0.344156</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.354078</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>0.363558</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0.372577</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>0.324795</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>0.336824</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0.348606</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0.360058</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0.370937</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>0.128303</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>0.315368</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.329339</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.343169</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>0.356587</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0.369291</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0.128302</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
           <t>EQE (absolute), n_sub = n_SL = 1.51, ETL 200 nm / HTL 200 nm x3</t>
         </is>
       </c>

</xml_diff>